<commit_message>
Update projects change video
</commit_message>
<xml_diff>
--- a/UPDATE/Projects.xlsx
+++ b/UPDATE/Projects.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\site\UPDATE\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\naama lavee\Documents\site\UPDATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82D23C68-D91A-4552-892F-C178DA20163E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62FF68D6-731C-4727-A124-19E3672BE3F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -138,14 +138,6 @@
     <t>Roni Kalev / Shifra Milshtein</t>
   </si>
   <si>
-    <t xml:space="preserve">Text and theatrical direction - Dalit Milshtein
-Costumes - Michal Laor / Light design - Judy Kupferman 
-</t>
-  </si>
-  <si>
-    <t>https://youtu.be/xQSFbspSqgA?si=XA_n3uNZ0Y3JGbLp</t>
-  </si>
-  <si>
     <t>Irish pub</t>
   </si>
   <si>
@@ -252,6 +244,14 @@
   <si>
     <t>War Zone</t>
   </si>
+  <si>
+    <t>https://youtu.be/jaoDg6OCPow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Text and theatrical direction - Dalit Milshtein
+/ Costumes - Michal Laor / Light design - Judy Kupferman 
+</t>
+  </si>
 </sst>
 </file>
 
@@ -260,7 +260,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mmmm\ yyyy"/>
   </numFmts>
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -314,12 +314,6 @@
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
     </font>
     <font>
       <u/>
@@ -393,7 +387,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -431,21 +425,18 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -821,32 +812,32 @@
       <c r="Y3" s="2"/>
       <c r="Z3" s="2"/>
     </row>
-    <row r="4" spans="1:26" ht="75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
-      <c r="B4" s="7" t="s">
-        <v>28</v>
+      <c r="B4" s="12" t="s">
+        <v>34</v>
       </c>
-      <c r="C4" s="8" t="s">
-        <v>29</v>
+      <c r="C4" s="1" t="s">
+        <v>35</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="9" t="s">
-        <v>30</v>
+      <c r="E4" s="13" t="s">
+        <v>36</v>
       </c>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
-      <c r="H4" s="9" t="s">
-        <v>31</v>
+      <c r="H4" s="14" t="s">
+        <v>68</v>
       </c>
       <c r="I4" s="10">
-        <v>45413</v>
+        <v>46023</v>
       </c>
-      <c r="J4" s="11" t="s">
-        <v>32</v>
+      <c r="J4" s="6" t="s">
+        <v>67</v>
       </c>
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
@@ -865,32 +856,32 @@
       <c r="Y4" s="2"/>
       <c r="Z4" s="2"/>
     </row>
-    <row r="5" spans="1:26" ht="110.25" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:26" ht="75" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
-      <c r="B5" s="12" t="s">
-        <v>34</v>
+      <c r="B5" s="7" t="s">
+        <v>28</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>35</v>
+      <c r="C5" s="8" t="s">
+        <v>29</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E5" s="13" t="s">
-        <v>36</v>
+      <c r="E5" s="9" t="s">
+        <v>30</v>
       </c>
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
-      <c r="H5" s="14" t="s">
-        <v>37</v>
+      <c r="H5" s="9" t="s">
+        <v>31</v>
       </c>
       <c r="I5" s="10">
-        <v>46023</v>
+        <v>45413</v>
       </c>
-      <c r="J5" s="15" t="s">
-        <v>38</v>
+      <c r="J5" s="11" t="s">
+        <v>32</v>
       </c>
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
@@ -911,24 +902,24 @@
     </row>
     <row r="6" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
-      <c r="B6" s="16" t="s">
-        <v>40</v>
+      <c r="B6" s="15" t="s">
+        <v>38</v>
       </c>
       <c r="C6" s="1"/>
       <c r="D6" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E6" s="16"/>
-      <c r="F6" s="16"/>
-      <c r="G6" s="16"/>
-      <c r="H6" s="16"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
       <c r="I6" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
-      <c r="J6" s="17" t="s">
-        <v>42</v>
+      <c r="J6" s="16" t="s">
+        <v>40</v>
       </c>
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
@@ -948,25 +939,25 @@
       <c r="Z6" s="2"/>
     </row>
     <row r="7" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="18" t="s">
-        <v>43</v>
+      <c r="A7" s="17" t="s">
+        <v>41</v>
       </c>
-      <c r="B7" s="16" t="s">
-        <v>44</v>
+      <c r="B7" s="15" t="s">
+        <v>42</v>
       </c>
-      <c r="C7" s="16"/>
+      <c r="C7" s="15"/>
       <c r="D7" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E7" s="16"/>
-      <c r="F7" s="16"/>
-      <c r="G7" s="16"/>
-      <c r="H7" s="16"/>
+      <c r="E7" s="15"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="15"/>
       <c r="I7" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
-      <c r="J7" s="17" t="s">
-        <v>46</v>
+      <c r="J7" s="16" t="s">
+        <v>44</v>
       </c>
       <c r="K7" s="2"/>
       <c r="L7" s="2"/>
@@ -987,25 +978,25 @@
     </row>
     <row r="8" spans="1:26" ht="63.75" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
-      <c r="B8" s="19" t="s">
-        <v>47</v>
+      <c r="B8" s="18" t="s">
+        <v>45</v>
       </c>
-      <c r="C8" s="16"/>
+      <c r="C8" s="15"/>
       <c r="D8" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E8" s="16"/>
-      <c r="F8" s="16"/>
-      <c r="G8" s="16"/>
-      <c r="H8" s="16"/>
-      <c r="I8" s="16"/>
-      <c r="J8" s="20" t="s">
-        <v>48</v>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="15"/>
+      <c r="J8" s="19" t="s">
+        <v>46</v>
       </c>
       <c r="K8" s="11" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="L8" s="2"/>
       <c r="M8" s="2"/>
@@ -1024,29 +1015,29 @@
       <c r="Z8" s="2"/>
     </row>
     <row r="9" spans="1:26" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A9" s="18" t="s">
-        <v>50</v>
+      <c r="A9" s="17" t="s">
+        <v>48</v>
       </c>
-      <c r="B9" s="16" t="s">
-        <v>51</v>
+      <c r="B9" s="15" t="s">
+        <v>49</v>
       </c>
-      <c r="C9" s="16"/>
+      <c r="C9" s="15"/>
       <c r="D9" s="1" t="s">
         <v>23</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F9" s="16"/>
-      <c r="G9" s="16"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15"/>
       <c r="H9" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
-      <c r="J9" s="17" t="s">
-        <v>54</v>
+      <c r="J9" s="16" t="s">
+        <v>52</v>
       </c>
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
@@ -1066,27 +1057,27 @@
       <c r="Z9" s="2"/>
     </row>
     <row r="10" spans="1:26" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A10" s="21" t="s">
-        <v>55</v>
+      <c r="A10" s="20" t="s">
+        <v>53</v>
       </c>
-      <c r="B10" s="22" t="s">
-        <v>56</v>
+      <c r="B10" s="21" t="s">
+        <v>54</v>
       </c>
-      <c r="C10" s="16"/>
+      <c r="C10" s="15"/>
       <c r="D10" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E10" s="16"/>
-      <c r="F10" s="16"/>
-      <c r="G10" s="16"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="15"/>
       <c r="H10" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
-      <c r="J10" s="17" t="s">
-        <v>59</v>
+      <c r="J10" s="16" t="s">
+        <v>57</v>
       </c>
       <c r="K10" s="2"/>
       <c r="L10" s="2"/>
@@ -1105,26 +1096,26 @@
       <c r="Y10" s="2"/>
       <c r="Z10" s="2"/>
     </row>
-    <row r="11" spans="1:26" ht="51" x14ac:dyDescent="0.2">
-      <c r="A11" s="23" t="s">
+    <row r="11" spans="1:26" ht="52.5" x14ac:dyDescent="0.3">
+      <c r="A11" s="22" t="s">
+        <v>58</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="D11" s="15"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="15"/>
+      <c r="I11" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="J11" s="16" t="s">
         <v>62</v>
-      </c>
-      <c r="D11" s="16"/>
-      <c r="E11" s="16"/>
-      <c r="F11" s="16"/>
-      <c r="G11" s="16"/>
-      <c r="H11" s="16"/>
-      <c r="I11" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="J11" s="17" t="s">
-        <v>64</v>
       </c>
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
@@ -1145,22 +1136,22 @@
     </row>
     <row r="12" spans="1:26" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
-      <c r="C12" s="16"/>
+      <c r="C12" s="15"/>
       <c r="D12" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E12" s="16"/>
-      <c r="F12" s="16"/>
-      <c r="G12" s="16"/>
-      <c r="H12" s="16"/>
-      <c r="I12" s="16"/>
-      <c r="J12" s="17" t="s">
-        <v>67</v>
+      <c r="E12" s="15"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="15"/>
+      <c r="I12" s="15"/>
+      <c r="J12" s="16" t="s">
+        <v>65</v>
       </c>
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
@@ -28875,16 +28866,15 @@
   <hyperlinks>
     <hyperlink ref="J2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="J3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="J4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="J5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="J6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="J7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="J8" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="K8" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="J9" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="J10" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="J11" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="J12" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="J5" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="J6" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="J7" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="J8" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="K8" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="J9" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="J10" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="J11" r:id="rId10" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="J12" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>